<commit_message>
data: Trading Economics xlsx API 증분 갱신 (2026-09-11) [A-248]
</commit_message>
<xml_diff>
--- a/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
+++ b/data/raw/Trading Economics/Markets/Commodities/Industrial/2019~2026_Urea_CBOT_USD Per Ton.xlsx
@@ -50531,7 +50531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -53742,14 +53742,25 @@
       <c r="H140" s="10" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" t="n">
+      <c r="A141" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B141" t="n">
+      <c r="B141" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F141" t="n">
+      <c r="F141" s="0" t="n">
         <v>450.25</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>9</v>
+      </c>
+      <c r="B142" t="n">
+        <v>11</v>
+      </c>
+      <c r="F142" t="n">
+        <v>450.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>